<commit_message>
Make Cindy baseline builders configurable and reproducible & make it cleaner
Update builder_pods.py to support reproducible baseline generation for Cindy Scenario 2 and Scenario 3.

Changes:

Add seeded SKU-order randomization within ABC classes for Scenario 2.
Add seeded SKU-order randomization within ABC classes for Scenario 3.
Add dynamic mixed-class slot planning for Scenario 3 instead of fixed 12/21/7 class zones.
Add minimum_inventory as a supported baseline target source.
Add robust parsing for semicolon-separated minimum_inventory.csv with comma decimals.
Preserve partial final-slot quantities when splitting SKU inventory across slots.
Route scenario2_baseline and scenario3_baseline to their correct builder functions.
Pass pod ID shuffle options into prepare_inputs() to support randomized physical pod mapping.

This patch does not change the optimizer, RMFS runtime logic, experiment SKU universe, or prepare_static_21day_inputs.py.
</commit_message>
<xml_diff>
--- a/summary_result.csv.xlsx
+++ b/summary_result.csv.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lukman-rmfs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ITB\Tugas Akhir\_full_postt_parallel_runs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D8F7B92-B268-4B12-9A67-700C6B367AF3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BBB373-8FB8-471B-9D23-776C1C3132D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="8736" xr2:uid="{B90FB510-2F72-4967-9247-29B5AFC05068}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B90FB510-2F72-4967-9247-29B5AFC05068}"/>
   </bookViews>
   <sheets>
     <sheet name="工作表1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="53">
   <si>
     <t>scenario</t>
   </si>
@@ -136,19 +147,73 @@
   </si>
   <si>
     <t>Cindy Scenario 1</t>
+  </si>
+  <si>
+    <t>energy_per_sim_hour </t>
+  </si>
+  <si>
+    <t>97,572.06</t>
+  </si>
+  <si>
+    <t>98,446.35</t>
+  </si>
+  <si>
+    <t>95,396.43</t>
+  </si>
+  <si>
+    <t>99,560.50</t>
+  </si>
+  <si>
+    <t>energy per delivered line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">variable_energy_per_delivered_line </t>
+  </si>
+  <si>
+    <t xml:space="preserve">energy_per_pod_visit </t>
+  </si>
+  <si>
+    <t>5,728.00</t>
+  </si>
+  <si>
+    <t>5,618.41</t>
+  </si>
+  <si>
+    <t>5,428.70</t>
+  </si>
+  <si>
+    <t>6,053.62</t>
+  </si>
+  <si>
+    <t>8,541.01</t>
+  </si>
+  <si>
+    <t>8,497.05</t>
+  </si>
+  <si>
+    <t>8,315.63</t>
+  </si>
+  <si>
+    <t>9,142.42</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF1F2328"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -171,11 +236,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="一般" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -191,9 +258,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 佈景主題">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -231,7 +298,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -337,7 +404,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -479,7 +546,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -487,10 +554,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1CA5ABB-DD05-4CB9-B007-D4809B060B77}">
-  <dimension ref="A1:AF5"/>
+  <dimension ref="A1:AJ5"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.3984375" customWidth="1"/>
+    <col min="2" max="2" width="10.59765625" customWidth="1"/>
+    <col min="29" max="29" width="21.59765625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="23.59765625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="28.796875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.296875" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="15" customWidth="1"/>
+    <col min="34" max="34" width="12.796875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -587,8 +664,20 @@
       <c r="AF1" t="s">
         <v>31</v>
       </c>
+      <c r="AG1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>44</v>
+      </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -685,8 +774,20 @@
       <c r="AF2">
         <v>1492.57278871536</v>
       </c>
+      <c r="AG2" t="s">
+        <v>38</v>
+      </c>
+      <c r="AH2" s="2">
+        <v>6546.74</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>49</v>
+      </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -783,8 +884,20 @@
       <c r="AF3">
         <v>1100.5707824230101</v>
       </c>
+      <c r="AG3" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH3" s="2">
+        <v>6426.87</v>
+      </c>
+      <c r="AI3" t="s">
+        <v>46</v>
+      </c>
+      <c r="AJ3" t="s">
+        <v>50</v>
+      </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -881,8 +994,20 @@
       <c r="AF4">
         <v>1512.67025494575</v>
       </c>
+      <c r="AG4" t="s">
+        <v>40</v>
+      </c>
+      <c r="AH4">
+        <v>6230.21</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AJ4" t="s">
+        <v>51</v>
+      </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -978,6 +1103,18 @@
       </c>
       <c r="AF5">
         <v>1590.726015</v>
+      </c>
+      <c r="AG5" t="s">
+        <v>41</v>
+      </c>
+      <c r="AH5" s="2">
+        <v>6853.99</v>
+      </c>
+      <c r="AI5" t="s">
+        <v>48</v>
+      </c>
+      <c r="AJ5" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>